<commit_message>
Added git link to the form
</commit_message>
<xml_diff>
--- a/Self Assessment Form - IUM-TWEB.xlsx
+++ b/Self Assessment Form - IUM-TWEB.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\Desktop\Uni\3° anno\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\Desktop\Uni\3° anno\Footbal-Web-Page\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7976E306-E54F-49EF-9734-94CB505647EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B2F59BA-A9B0-490B-A1B9-A35C0E6A56D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6990" yWindow="0" windowWidth="23805" windowHeight="19260" xr2:uid="{9384817B-0988-A24F-9D66-74DAD74AC274}"/>
+    <workbookView xWindow="12990" yWindow="945" windowWidth="24405" windowHeight="19260" xr2:uid="{9384817B-0988-A24F-9D66-74DAD74AC274}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="66">
   <si>
     <t>Team Name</t>
   </si>
@@ -250,6 +250,13 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>https://github.com/B-u-b-y/Jupiter-Notebooks
+https://github.com/B-u-b-y/Footbal-Web-Page
+https://github.com/B-u-b-y/Server-Flask
+https://github.com/B-u-b-y/Server_Express
+https://github.com/B-u-b-y/Spring-Boot-Server</t>
   </si>
 </sst>
 </file>
@@ -555,15 +562,6 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -575,6 +573,15 @@
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -902,20 +909,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="37" customFormat="1" ht="95.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
     </row>
     <row r="2" spans="1:5" s="37" customFormat="1" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -969,11 +976,13 @@
       <c r="B10" s="27"/>
       <c r="C10" s="7"/>
     </row>
-    <row r="11" spans="1:5" ht="33.75" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="159" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="24"/>
+      <c r="B11" s="24" t="s">
+        <v>65</v>
+      </c>
       <c r="C11" s="39" t="s">
         <v>47</v>
       </c>
@@ -1183,7 +1192,7 @@
       <c r="C38" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D38" s="44" t="s">
+      <c r="D38" s="41" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1233,7 +1242,7 @@
       <c r="C46" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D46" s="45" t="s">
+      <c r="D46" s="42" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1310,7 +1319,7 @@
       <c r="C55" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D55" s="43" t="s">
+      <c r="D55" s="40" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1360,7 +1369,7 @@
       <c r="C60" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D60" s="43" t="s">
+      <c r="D60" s="40" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1400,7 +1409,7 @@
       <c r="C68" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D68" s="43" t="s">
+      <c r="D68" s="40" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1457,7 +1466,7 @@
       <c r="A76" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="B76" s="46">
+      <c r="B76" s="43">
         <v>1</v>
       </c>
       <c r="C76" s="4"/>

</xml_diff>